<commit_message>
kurir, change variabel, optimasi
</commit_message>
<xml_diff>
--- a/template_adjacency_20node.xlsx
+++ b/template_adjacency_20node.xlsx
@@ -435,14 +435,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2. Sheet 'Paket': isi data paket per node. Node asal/deposit: Volume=0, Prioritas=0, Deadline=0.</t>
+          <t>2. Sheet 'Paket': isi data paket. Asal = Depot asal pengiriman paket (default: A). Tujuan = Node tujuan paket.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>3. Node asal di aplikasi = baris pertama di sheet Paket (Node1) atau pilih manual di sidebar.</t>
+          <t>3. Untuk baris Depot Asal sendiri (Tujuan = A): Berat=0, Prioritas=0, Deadline=0.</t>
         </is>
       </c>
     </row>
@@ -456,7 +456,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>5. Minimal 20 node sudah disediakan, bisa ditambah/diubah namanya asalkan konsisten antar sheet.</t>
+          <t>5. Template berisi 20 lokasi: A s/d T.</t>
         </is>
       </c>
     </row>
@@ -477,109 +477,109 @@
     <row r="1">
       <c r="B1" t="inlineStr">
         <is>
-          <t>Node1</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Node2</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Node3</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Node4</t>
+          <t>D</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Node5</t>
+          <t>E</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Node6</t>
+          <t>F</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Node7</t>
+          <t>G</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Node8</t>
+          <t>H</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>Node9</t>
+          <t>I</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>Node10</t>
+          <t>J</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>Node11</t>
+          <t>K</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>Node12</t>
+          <t>L</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>Node13</t>
+          <t>M</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>Node14</t>
+          <t>N</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>Node15</t>
+          <t>O</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>Node16</t>
+          <t>P</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>Node17</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>Node18</t>
+          <t>R</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>Node19</t>
+          <t>S</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>Node20</t>
+          <t>T</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Node1</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -646,7 +646,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Node2</t>
+          <t>B</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -713,7 +713,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Node3</t>
+          <t>C</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -780,7 +780,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Node4</t>
+          <t>D</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -847,7 +847,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Node5</t>
+          <t>E</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -914,7 +914,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Node6</t>
+          <t>F</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -981,7 +981,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Node7</t>
+          <t>G</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -1048,7 +1048,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Node8</t>
+          <t>H</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -1115,7 +1115,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Node9</t>
+          <t>I</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -1182,7 +1182,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Node10</t>
+          <t>J</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -1249,7 +1249,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Node11</t>
+          <t>K</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -1316,7 +1316,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Node12</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1383,7 +1383,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Node13</t>
+          <t>M</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -1450,7 +1450,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Node14</t>
+          <t>N</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1517,7 +1517,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Node15</t>
+          <t>O</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -1584,7 +1584,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Node16</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1651,7 +1651,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Node17</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -1718,7 +1718,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Node18</t>
+          <t>R</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1785,7 +1785,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Node19</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1852,7 +1852,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Node20</t>
+          <t>T</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1927,26 +1927,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Node</t>
+          <t>Asal</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Volume (m2)</t>
+          <t>Tujuan</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Berat (kg)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Prioritas (1-3)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Deadline (jam)</t>
         </is>
@@ -1955,11 +1960,13 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Node1</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>0</v>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -1967,308 +1974,406 @@
       <c r="D2" t="n">
         <v>0</v>
       </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Node2</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
         <v>4</v>
-      </c>
-      <c r="C3" t="n">
-        <v>2</v>
       </c>
       <c r="D3" t="n">
         <v>2</v>
       </c>
+      <c r="E3" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Node3</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
         <v>5</v>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="n">
         <v>3</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>2.5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Node4</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
         <v>6</v>
       </c>
-      <c r="C5" t="n">
+      <c r="D5" t="n">
         <v>1</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Node5</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
         <v>7</v>
       </c>
-      <c r="C6" t="n">
+      <c r="D6" t="n">
         <v>2</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>3.5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Node6</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>3</v>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
       </c>
       <c r="C7" t="n">
         <v>3</v>
       </c>
       <c r="D7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Node7</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
         <v>4</v>
       </c>
-      <c r="C8" t="n">
+      <c r="D8" t="n">
         <v>1</v>
       </c>
-      <c r="D8" t="n">
+      <c r="E8" t="n">
         <v>1.5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Node8</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
         <v>5</v>
-      </c>
-      <c r="C9" t="n">
-        <v>2</v>
       </c>
       <c r="D9" t="n">
         <v>2</v>
       </c>
+      <c r="E9" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Node9</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
         <v>6</v>
       </c>
-      <c r="C10" t="n">
+      <c r="D10" t="n">
         <v>3</v>
       </c>
-      <c r="D10" t="n">
+      <c r="E10" t="n">
         <v>2.5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Node10</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
         <v>7</v>
       </c>
-      <c r="C11" t="n">
+      <c r="D11" t="n">
         <v>1</v>
       </c>
-      <c r="D11" t="n">
+      <c r="E11" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Node11</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
         <v>3</v>
       </c>
-      <c r="C12" t="n">
+      <c r="D12" t="n">
         <v>2</v>
       </c>
-      <c r="D12" t="n">
+      <c r="E12" t="n">
         <v>3.5</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Node12</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
         <v>4</v>
       </c>
-      <c r="C13" t="n">
+      <c r="D13" t="n">
         <v>3</v>
       </c>
-      <c r="D13" t="n">
+      <c r="E13" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Node13</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
         <v>5</v>
       </c>
-      <c r="C14" t="n">
+      <c r="D14" t="n">
         <v>1</v>
       </c>
-      <c r="D14" t="n">
+      <c r="E14" t="n">
         <v>1.5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Node14</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
         <v>6</v>
-      </c>
-      <c r="C15" t="n">
-        <v>2</v>
       </c>
       <c r="D15" t="n">
         <v>2</v>
       </c>
+      <c r="E15" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Node15</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
         <v>7</v>
       </c>
-      <c r="C16" t="n">
+      <c r="D16" t="n">
         <v>3</v>
       </c>
-      <c r="D16" t="n">
+      <c r="E16" t="n">
         <v>2.5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Node16</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
         <v>3</v>
       </c>
-      <c r="C17" t="n">
+      <c r="D17" t="n">
         <v>1</v>
       </c>
-      <c r="D17" t="n">
+      <c r="E17" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Node17</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
         <v>4</v>
       </c>
-      <c r="C18" t="n">
+      <c r="D18" t="n">
         <v>2</v>
       </c>
-      <c r="D18" t="n">
+      <c r="E18" t="n">
         <v>3.5</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Node18</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
         <v>5</v>
       </c>
-      <c r="C19" t="n">
+      <c r="D19" t="n">
         <v>3</v>
       </c>
-      <c r="D19" t="n">
+      <c r="E19" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Node19</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
         <v>6</v>
       </c>
-      <c r="C20" t="n">
+      <c r="D20" t="n">
         <v>1</v>
       </c>
-      <c r="D20" t="n">
+      <c r="E20" t="n">
         <v>1.5</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Node20</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
         <v>7</v>
       </c>
-      <c r="C21" t="n">
+      <c r="D21" t="n">
         <v>2</v>
       </c>
-      <c r="D21" t="n">
+      <c r="E21" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>